<commit_message>
chore: update word list in Words.xlsx
Updated the Words.xlsx binary file, likely adding or modifying
word entries used in the WordGuessing game.
</commit_message>
<xml_diff>
--- a/Words.xlsx
+++ b/Words.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ADisk\Project\WordGuessing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A6597D0-5694-494B-80B8-B0FBE46B3F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C75C74-7BEC-40E4-B77F-98576B98F4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14835" yWindow="-12855" windowWidth="19200" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Word</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -61,6 +61,15 @@
     <t xml:space="preserve"> the process of extracting information that is 
 essential, while ignoring what is not relevant, for the 
 provision of a solution.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Acceptance testing</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>the testing of a completed program to 
+prove to the customer that it works as required.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -389,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.4140625" customWidth="1"/>
@@ -428,6 +437,14 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="1:2" ht="56" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add Quit Game button and update README
</commit_message>
<xml_diff>
--- a/Words.xlsx
+++ b/Words.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ADisk\Project\WordGuessing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C75C74-7BEC-40E4-B77F-98576B98F4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF7E7A2-8E98-435E-8FEA-169BE4DAC052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14835" yWindow="-12855" windowWidth="19200" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9675" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>Word</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -35,41 +35,219 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>A* algorithm</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>An algorithm that finds the shortest route 
-between nodes or vertices but uses an additional heuristic 
-approach to achieve better performance than Dijkstra’s 
-algorithm.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Abnormal test data </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>test data that should be rejected by a program</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Abstraction</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> the process of extracting information that is 
-essential, while ignoring what is not relevant, for the 
-provision of a solution.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Acceptance testing</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>the testing of a completed program to 
-prove to the customer that it works as required.</t>
+    <t>Random access memory (RAM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>primary memory unit 
+that can be written to and read from.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Read-only memory (ROM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Programmable ROM (PROM) </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> type of ROM chip that 
+can be programmed once.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> primary memory unit that 
+can only be read from.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Erasable PROM (EPROM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> type of ROM that can be 
+programmed more than once</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hard disk drive (HDD)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>type of magnetic storage device 
+that uses spinning disks.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Latency</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>the lag in a system</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fragmented</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> storage of data in non-consecutive sectors</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Solid state drive (SSD)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>storage media with no moving 
+parts that relies on movement of electrons.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Electronically erasable programmable read-only 
+memory (EEPROM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> read-only (ROM) chip that can 
+be modified by the user, which can then be erased and 
+written to repeatedly </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Flash memory </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>a type of EEPROM, particularly suited 
+to use in drives such as SSDs, memory cards and 
+memory sticks</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Optical storage </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Birefringence </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>a reading problem with DVDs caused 
+by refraction of laser light into two beams.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CDs, DVDs and Blu-rayTM discs that 
+use laser light to read and write data.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Digital to analogue converter (DAC) </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> needed to 
+convert digital data into electric currents that can drive 
+motors, actuators and relays, for example.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Analogue to digital converter (ADC) </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>needed to 
+convert analogue data (read from sensors, for example) 
+into a form understood by a computer.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Screen resolution</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>number of pixels in the horizontal 
+and vertical directions on a television/computer screen.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Capacitive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>type of touch screen technology based 
+on glass layers forming a capacitor, where fingers 
+touching the screen cause a change in the electric field.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Resistive</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>type of touch screen technology. When 
+a finger touches the screen, the glass layer touches 
+the plastic layer, completing the circuit and causing a 
+current to flow at that point.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sensor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>input device that reads physical data from its 
+surroundings.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Logic gates</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>electronic circuits which rely on 
+‘on/off’ logic.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Logic circuit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>a combination of logic gates 
+and designed to carry out a particular task.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Truth table </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">a method of checking the output from 
+a logic circuit. They use all the possible binary input 
+combinations depending on the number of inputs; </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Boolean algebra </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>a form of algebra linked to logic 
+circuits and based on TRUE and FALSE.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OLED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>uses movement of electrons 
+between cathode and anode to produce an on-screen 
+image. It generates its own light so no back lighting 
+required.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -398,10 +576,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.4140625" customWidth="1"/>
+    <col min="1" max="1" width="31.5" customWidth="1"/>
     <col min="2" max="2" width="28.1640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -413,7 +591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="98" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="42" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -421,28 +599,180 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="28" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="70" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="56" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:2" ht="28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="28" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="28" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="42" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="56" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="70" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="56" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="56" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="70" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="70" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="42" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="84" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="98" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="42" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="28" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="42" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="84" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="42" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="84" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>